<commit_message>
first successful contact with ai
</commit_message>
<xml_diff>
--- a/TestDocuments/Массив ответов 001.xlsx
+++ b/TestDocuments/Массив ответов 001.xlsx
@@ -1,15 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c.dorzhieva\Downloads\ЭН\ЭН\2025_10_23-2025_12_21_Электронное наставничество\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11100" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11100" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Промежуточный тест 1" sheetId="1" r:id="rId1"/>
@@ -18,7 +13,7 @@
     <sheet name="Промежуточный тест 4" sheetId="4" r:id="rId4"/>
     <sheet name="Итоговый тест" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -1150,7 +1145,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="11">
     <numFmt numFmtId="164" formatCode="d\.m\.yyyy\ h:mm"/>
     <numFmt numFmtId="165" formatCode="d\.m\.yyyy\ hh:m"/>
@@ -1164,7 +1159,7 @@
     <numFmt numFmtId="173" formatCode="0.0"/>
     <numFmt numFmtId="174" formatCode="0.#"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -1319,7 +1314,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1371,7 +1366,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1565,16 +1560,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:FP20"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" customWidth="1"/>
@@ -1724,7 +1719,7 @@
     <col min="171" max="172" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:172" ht="25.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1990,7 +1985,7 @@
       <c r="FO1" s="1"/>
       <c r="FP1" s="1"/>
     </row>
-    <row r="2" spans="1:172" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:172">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2500,7 +2495,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:172" ht="25.5">
       <c r="A3" s="3">
         <v>20251022001</v>
       </c>
@@ -2802,7 +2797,7 @@
       <c r="FO3" s="2"/>
       <c r="FP3" s="2"/>
     </row>
-    <row r="4" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:172" ht="25.5">
       <c r="A4" s="2" t="s">
         <v>55</v>
       </c>
@@ -3104,7 +3099,7 @@
       <c r="FO4" s="2"/>
       <c r="FP4" s="2"/>
     </row>
-    <row r="5" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:172" ht="25.5">
       <c r="A5" s="2" t="s">
         <v>55</v>
       </c>
@@ -3376,7 +3371,7 @@
       <c r="FO5" s="2"/>
       <c r="FP5" s="2"/>
     </row>
-    <row r="6" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:172" ht="25.5">
       <c r="A6" s="3">
         <v>20251021004</v>
       </c>
@@ -3678,7 +3673,7 @@
       <c r="FO6" s="2"/>
       <c r="FP6" s="2"/>
     </row>
-    <row r="7" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:172" ht="25.5">
       <c r="A7" s="3">
         <v>20251024002</v>
       </c>
@@ -3980,7 +3975,7 @@
       <c r="FO7" s="2"/>
       <c r="FP7" s="2"/>
     </row>
-    <row r="8" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:172" ht="25.5">
       <c r="A8" s="3">
         <v>20251021007</v>
       </c>
@@ -4282,7 +4277,7 @@
       <c r="FO8" s="2"/>
       <c r="FP8" s="2"/>
     </row>
-    <row r="9" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:172" ht="25.5">
       <c r="A9" s="3">
         <v>20251022001</v>
       </c>
@@ -4554,7 +4549,7 @@
       <c r="FO9" s="2"/>
       <c r="FP9" s="2"/>
     </row>
-    <row r="10" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:172" ht="25.5">
       <c r="A10" s="3">
         <v>20251024001</v>
       </c>
@@ -4856,7 +4851,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:172" ht="25.5">
       <c r="A11" s="3">
         <v>20251024001</v>
       </c>
@@ -5128,7 +5123,7 @@
       <c r="FO11" s="2"/>
       <c r="FP11" s="2"/>
     </row>
-    <row r="12" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:172" ht="25.5">
       <c r="A12" s="3">
         <v>20251021008</v>
       </c>
@@ -5430,7 +5425,7 @@
       <c r="FO12" s="2"/>
       <c r="FP12" s="2"/>
     </row>
-    <row r="13" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:172" ht="25.5">
       <c r="A13" s="3">
         <v>20251021008</v>
       </c>
@@ -5732,7 +5727,7 @@
       <c r="FO13" s="2"/>
       <c r="FP13" s="2"/>
     </row>
-    <row r="14" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:172" ht="25.5">
       <c r="A14" s="3">
         <v>20251021003</v>
       </c>
@@ -6034,7 +6029,7 @@
       <c r="FO14" s="2"/>
       <c r="FP14" s="2"/>
     </row>
-    <row r="15" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:172" ht="25.5">
       <c r="A15" s="3">
         <v>20251021003</v>
       </c>
@@ -6336,7 +6331,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:172" ht="25.5">
       <c r="A16" s="3">
         <v>20251021008</v>
       </c>
@@ -6608,7 +6603,7 @@
       <c r="FO16" s="2"/>
       <c r="FP16" s="2"/>
     </row>
-    <row r="17" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:172" ht="25.5">
       <c r="A17" s="3">
         <v>20251021001</v>
       </c>
@@ -6910,7 +6905,7 @@
       <c r="FO17" s="2"/>
       <c r="FP17" s="2"/>
     </row>
-    <row r="18" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:172" ht="25.5">
       <c r="A18" s="3">
         <v>20251021001</v>
       </c>
@@ -7182,7 +7177,7 @@
       <c r="FO18" s="2"/>
       <c r="FP18" s="2"/>
     </row>
-    <row r="19" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:172" ht="25.5">
       <c r="A19" s="3">
         <v>20251021002</v>
       </c>
@@ -7484,7 +7479,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="20" spans="1:172" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:172" ht="25.5">
       <c r="A20" s="2" t="s">
         <v>119</v>
       </c>
@@ -7792,9 +7787,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:FD22"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" customWidth="1"/>
@@ -7922,7 +7917,7 @@
     <col min="159" max="160" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:160" ht="25.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8170,7 +8165,7 @@
       <c r="FC1" s="1"/>
       <c r="FD1" s="1"/>
     </row>
-    <row r="2" spans="1:160" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:160">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -8644,7 +8639,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:160" ht="25.5">
       <c r="A3" s="3">
         <v>20251022001</v>
       </c>
@@ -8934,7 +8929,7 @@
       <c r="FC3" s="2"/>
       <c r="FD3" s="2"/>
     </row>
-    <row r="4" spans="1:160" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:160">
       <c r="A4" s="3">
         <v>20251022001</v>
       </c>
@@ -9224,7 +9219,7 @@
       <c r="FC4" s="2"/>
       <c r="FD4" s="2"/>
     </row>
-    <row r="5" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:160" ht="25.5">
       <c r="A5" s="2" t="s">
         <v>55</v>
       </c>
@@ -9514,7 +9509,7 @@
       <c r="FC5" s="2"/>
       <c r="FD5" s="2"/>
     </row>
-    <row r="6" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:160" ht="25.5">
       <c r="A6" s="3">
         <v>20251022001</v>
       </c>
@@ -9804,7 +9799,7 @@
       <c r="FC6" s="2"/>
       <c r="FD6" s="2"/>
     </row>
-    <row r="7" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:160" ht="25.5">
       <c r="A7" s="3">
         <v>20251024002</v>
       </c>
@@ -10094,7 +10089,7 @@
       <c r="FC7" s="2"/>
       <c r="FD7" s="2"/>
     </row>
-    <row r="8" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:160" ht="25.5">
       <c r="A8" s="3">
         <v>20251024002</v>
       </c>
@@ -10354,7 +10349,7 @@
       <c r="FC8" s="2"/>
       <c r="FD8" s="2"/>
     </row>
-    <row r="9" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:160" ht="25.5">
       <c r="A9" s="3">
         <v>20251021004</v>
       </c>
@@ -10644,7 +10639,7 @@
       <c r="FC9" s="2"/>
       <c r="FD9" s="2"/>
     </row>
-    <row r="10" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:160" ht="25.5">
       <c r="A10" s="3">
         <v>20251022001</v>
       </c>
@@ -10904,7 +10899,7 @@
       <c r="FC10" s="2"/>
       <c r="FD10" s="2"/>
     </row>
-    <row r="11" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:160" ht="25.5">
       <c r="A11" s="3">
         <v>20251024001</v>
       </c>
@@ -11194,7 +11189,7 @@
       <c r="FC11" s="2"/>
       <c r="FD11" s="2"/>
     </row>
-    <row r="12" spans="1:160" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:160">
       <c r="A12" s="3">
         <v>20251021008</v>
       </c>
@@ -11484,7 +11479,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="13" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:160" ht="25.5">
       <c r="A13" s="3">
         <v>20251021003</v>
       </c>
@@ -11774,7 +11769,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="14" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:160" ht="25.5">
       <c r="A14" s="3">
         <v>20251021003</v>
       </c>
@@ -12038,7 +12033,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="15" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:160" ht="25.5">
       <c r="A15" s="3">
         <v>20251021001</v>
       </c>
@@ -12328,7 +12323,7 @@
       <c r="FC15" s="2"/>
       <c r="FD15" s="2"/>
     </row>
-    <row r="16" spans="1:160" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:160">
       <c r="A16" s="3">
         <v>20251021001</v>
       </c>
@@ -12588,7 +12583,7 @@
       <c r="FC16" s="2"/>
       <c r="FD16" s="2"/>
     </row>
-    <row r="17" spans="1:160" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:160">
       <c r="A17" s="3">
         <v>20251021002</v>
       </c>
@@ -12878,7 +12873,7 @@
       <c r="FC17" s="2"/>
       <c r="FD17" s="2"/>
     </row>
-    <row r="18" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:160" ht="25.5">
       <c r="A18" s="2" t="s">
         <v>119</v>
       </c>
@@ -13168,7 +13163,7 @@
       <c r="FC18" s="2"/>
       <c r="FD18" s="2"/>
     </row>
-    <row r="19" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:160" ht="25.5">
       <c r="A19" s="2" t="s">
         <v>119</v>
       </c>
@@ -13458,7 +13453,7 @@
       <c r="FC19" s="2"/>
       <c r="FD19" s="2"/>
     </row>
-    <row r="20" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:160" ht="25.5">
       <c r="A20" s="2" t="s">
         <v>119</v>
       </c>
@@ -13748,7 +13743,7 @@
       <c r="FC20" s="2"/>
       <c r="FD20" s="2"/>
     </row>
-    <row r="21" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:160" ht="25.5">
       <c r="A21" s="2" t="s">
         <v>119</v>
       </c>
@@ -14038,7 +14033,7 @@
       <c r="FC21" s="2"/>
       <c r="FD21" s="2"/>
     </row>
-    <row r="22" spans="1:160" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:160" ht="25.5">
       <c r="A22" s="3">
         <v>20251021007</v>
       </c>
@@ -14334,9 +14329,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:EF16"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" customWidth="1"/>
@@ -14452,7 +14447,7 @@
     <col min="135" max="136" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:136" ht="25.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -14664,7 +14659,7 @@
       <c r="EE1" s="1"/>
       <c r="EF1" s="1"/>
     </row>
-    <row r="2" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:136">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -15066,7 +15061,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:136" ht="25.5">
       <c r="A3" s="2" t="s">
         <v>55</v>
       </c>
@@ -15332,7 +15327,7 @@
       <c r="EE3" s="2"/>
       <c r="EF3" s="2"/>
     </row>
-    <row r="4" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:136">
       <c r="A4" s="3">
         <v>20251022001</v>
       </c>
@@ -15598,7 +15593,7 @@
       <c r="EE4" s="2"/>
       <c r="EF4" s="2"/>
     </row>
-    <row r="5" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:136" ht="25.5">
       <c r="A5" s="3">
         <v>20251024002</v>
       </c>
@@ -15864,7 +15859,7 @@
       <c r="EE5" s="2"/>
       <c r="EF5" s="2"/>
     </row>
-    <row r="6" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:136" ht="25.5">
       <c r="A6" s="3">
         <v>20251021004</v>
       </c>
@@ -16130,7 +16125,7 @@
       <c r="EE6" s="2"/>
       <c r="EF6" s="2"/>
     </row>
-    <row r="7" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:136">
       <c r="A7" s="3">
         <v>20251022001</v>
       </c>
@@ -16366,7 +16361,7 @@
       <c r="EE7" s="2"/>
       <c r="EF7" s="2"/>
     </row>
-    <row r="8" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:136" ht="25.5">
       <c r="A8" s="3">
         <v>20251024001</v>
       </c>
@@ -16632,7 +16627,7 @@
       <c r="EE8" s="2"/>
       <c r="EF8" s="2"/>
     </row>
-    <row r="9" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:136" ht="25.5">
       <c r="A9" s="3">
         <v>20251021003</v>
       </c>
@@ -16898,7 +16893,7 @@
       <c r="EE9" s="2"/>
       <c r="EF9" s="2"/>
     </row>
-    <row r="10" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:136" ht="25.5">
       <c r="A10" s="3">
         <v>20251021008</v>
       </c>
@@ -17164,7 +17159,7 @@
       <c r="EE10" s="2"/>
       <c r="EF10" s="2"/>
     </row>
-    <row r="11" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:136">
       <c r="A11" s="3">
         <v>20251021003</v>
       </c>
@@ -17400,7 +17395,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="12" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:136">
       <c r="A12" s="3">
         <v>20251021001</v>
       </c>
@@ -17666,7 +17661,7 @@
       <c r="EE12" s="2"/>
       <c r="EF12" s="2"/>
     </row>
-    <row r="13" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:136">
       <c r="A13" s="3">
         <v>20251021002</v>
       </c>
@@ -17932,7 +17927,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="14" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:136">
       <c r="A14" s="3">
         <v>20251021002</v>
       </c>
@@ -18198,7 +18193,7 @@
       <c r="EE14" s="2"/>
       <c r="EF14" s="2"/>
     </row>
-    <row r="15" spans="1:136" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:136" ht="25.5">
       <c r="A15" s="2" t="s">
         <v>119</v>
       </c>
@@ -18464,7 +18459,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="16" spans="1:136" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:136">
       <c r="A16" s="3">
         <v>20251021007</v>
       </c>
@@ -18736,9 +18731,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:CN18"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" customWidth="1"/>
@@ -18812,7 +18807,7 @@
     <col min="91" max="92" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:92">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -18958,7 +18953,7 @@
       <c r="CM1" s="1"/>
       <c r="CN1" s="1"/>
     </row>
-    <row r="2" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:92">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -19228,7 +19223,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:92" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:92" ht="25.5">
       <c r="A3" s="2" t="s">
         <v>55</v>
       </c>
@@ -19450,7 +19445,7 @@
       <c r="CM3" s="2"/>
       <c r="CN3" s="2"/>
     </row>
-    <row r="4" spans="1:92" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:92" ht="25.5">
       <c r="A4" s="2" t="s">
         <v>55</v>
       </c>
@@ -19642,7 +19637,7 @@
       <c r="CM4" s="2"/>
       <c r="CN4" s="2"/>
     </row>
-    <row r="5" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:92">
       <c r="A5" s="3">
         <v>20251022001</v>
       </c>
@@ -19864,7 +19859,7 @@
       <c r="CM5" s="2"/>
       <c r="CN5" s="2"/>
     </row>
-    <row r="6" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:92">
       <c r="A6" s="3">
         <v>20251024002</v>
       </c>
@@ -20086,7 +20081,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="7" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:92">
       <c r="A7" s="3">
         <v>20251021004</v>
       </c>
@@ -20308,7 +20303,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="8" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:92">
       <c r="A8" s="3">
         <v>20251022001</v>
       </c>
@@ -20500,7 +20495,7 @@
       <c r="CM8" s="2"/>
       <c r="CN8" s="2"/>
     </row>
-    <row r="9" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:92">
       <c r="A9" s="3">
         <v>20251024001</v>
       </c>
@@ -20722,7 +20717,7 @@
       <c r="CM9" s="2"/>
       <c r="CN9" s="2"/>
     </row>
-    <row r="10" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:92">
       <c r="A10" s="3">
         <v>20251024001</v>
       </c>
@@ -20914,7 +20909,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="11" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:92">
       <c r="A11" s="3">
         <v>20251021003</v>
       </c>
@@ -21136,7 +21131,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="12" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:92">
       <c r="A12" s="3">
         <v>20251021003</v>
       </c>
@@ -21328,7 +21323,7 @@
       <c r="CM12" s="2"/>
       <c r="CN12" s="2"/>
     </row>
-    <row r="13" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:92">
       <c r="A13" s="3">
         <v>20251021008</v>
       </c>
@@ -21550,7 +21545,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="14" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:92">
       <c r="A14" s="3">
         <v>20251021001</v>
       </c>
@@ -21772,7 +21767,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="15" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:92">
       <c r="A15" s="3">
         <v>20251021001</v>
       </c>
@@ -21964,7 +21959,7 @@
       <c r="CM15" s="2"/>
       <c r="CN15" s="2"/>
     </row>
-    <row r="16" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:92">
       <c r="A16" s="3">
         <v>20251021002</v>
       </c>
@@ -22186,7 +22181,7 @@
       <c r="CM16" s="2"/>
       <c r="CN16" s="2"/>
     </row>
-    <row r="17" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:92">
       <c r="A17" s="2" t="s">
         <v>119</v>
       </c>
@@ -22408,7 +22403,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="18" spans="1:92" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:92">
       <c r="A18" s="3">
         <v>20251021007</v>
       </c>
@@ -22636,9 +22631,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:TP13"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" customWidth="1"/>
@@ -23063,7 +23058,7 @@
     <col min="535" max="536" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:536" ht="25.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -23875,7 +23870,7 @@
       <c r="TO1" s="1"/>
       <c r="TP1" s="1"/>
     </row>
-    <row r="2" spans="1:536" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:536">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -25477,7 +25472,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:536" ht="25.5">
       <c r="A3" s="2" t="s">
         <v>55</v>
       </c>
@@ -26423,7 +26418,7 @@
       <c r="TO3" s="2"/>
       <c r="TP3" s="2"/>
     </row>
-    <row r="4" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:536" ht="25.5">
       <c r="A4" s="3">
         <v>20251024002</v>
       </c>
@@ -27369,7 +27364,7 @@
       <c r="TO4" s="2"/>
       <c r="TP4" s="2"/>
     </row>
-    <row r="5" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:536" ht="25.5">
       <c r="A5" s="3">
         <v>20251021004</v>
       </c>
@@ -28315,7 +28310,7 @@
       <c r="TO5" s="2"/>
       <c r="TP5" s="2"/>
     </row>
-    <row r="6" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:536" ht="25.5">
       <c r="A6" s="3">
         <v>20251022001</v>
       </c>
@@ -29261,7 +29256,7 @@
       <c r="TO6" s="2"/>
       <c r="TP6" s="2"/>
     </row>
-    <row r="7" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:536" ht="25.5">
       <c r="A7" s="3">
         <v>20251024001</v>
       </c>
@@ -30207,7 +30202,7 @@
       <c r="TO7" s="2"/>
       <c r="TP7" s="2"/>
     </row>
-    <row r="8" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:536" ht="25.5">
       <c r="A8" s="3">
         <v>20251021003</v>
       </c>
@@ -31153,7 +31148,7 @@
       <c r="TO8" s="2"/>
       <c r="TP8" s="2"/>
     </row>
-    <row r="9" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:536" ht="25.5">
       <c r="A9" s="3">
         <v>20251021008</v>
       </c>
@@ -32099,7 +32094,7 @@
       <c r="TO9" s="2"/>
       <c r="TP9" s="2"/>
     </row>
-    <row r="10" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:536" ht="25.5">
       <c r="A10" s="3">
         <v>20251021001</v>
       </c>
@@ -33045,7 +33040,7 @@
       <c r="TO10" s="2"/>
       <c r="TP10" s="2"/>
     </row>
-    <row r="11" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:536" ht="25.5">
       <c r="A11" s="3">
         <v>20251021002</v>
       </c>
@@ -33991,7 +33986,7 @@
       <c r="TO11" s="2"/>
       <c r="TP11" s="2"/>
     </row>
-    <row r="12" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:536" ht="25.5">
       <c r="A12" s="2" t="s">
         <v>119</v>
       </c>
@@ -34937,7 +34932,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="13" spans="1:536" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:536" ht="25.5">
       <c r="A13" s="3">
         <v>20251021007</v>
       </c>

</xml_diff>